<commit_message>
fix(excel-import): smart sheet/header detection and prevent cloud sync from overwriting local imports
</commit_message>
<xml_diff>
--- a/HRM_Database_Normalized.xlsx
+++ b/HRM_Database_Normalized.xlsx
@@ -610,10 +610,10 @@
         <v>Kích hoạt</v>
       </c>
       <c r="H2" t="str">
-        <v>$2b$10$d0w1iLTS0jPGoh.tPo.7buuJSQlC9cCz5JWMZeP4umcO0RbPvTn8W</v>
+        <v>$2b$10$gACgAHs317llVz7hBkSzueTGLnn6In3w1Fvzk0kANlfXI1qg4InL2</v>
       </c>
       <c r="I2" t="str">
-        <v>2026-09-04T04:58:27.529Z</v>
+        <v>2026-09-04T07:13:08.637Z</v>
       </c>
     </row>
     <row r="3">
@@ -639,10 +639,10 @@
         <v>Kích hoạt</v>
       </c>
       <c r="H3" t="str">
-        <v>$2b$10$d0w1iLTS0jPGoh.tPo.7buuJSQlC9cCz5JWMZeP4umcO0RbPvTn8W</v>
+        <v>$2b$10$gACgAHs317llVz7hBkSzueTGLnn6In3w1Fvzk0kANlfXI1qg4InL2</v>
       </c>
       <c r="I3" t="str">
-        <v>2026-09-04T04:58:27.529Z</v>
+        <v>2026-09-04T07:13:08.637Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(persistence): synchronous batch export to google sheets on excel import to prevent data loss on reload
</commit_message>
<xml_diff>
--- a/HRM_Database_Normalized.xlsx
+++ b/HRM_Database_Normalized.xlsx
@@ -610,10 +610,10 @@
         <v>Kích hoạt</v>
       </c>
       <c r="H2" t="str">
-        <v>$2b$10$gACgAHs317llVz7hBkSzueTGLnn6In3w1Fvzk0kANlfXI1qg4InL2</v>
+        <v>$2b$10$XSv.yrA1Pj8MUts1XMIYcuxvqv6rMCnq8C7kxgIp5j/tv1gZ4x4Fu</v>
       </c>
       <c r="I2" t="str">
-        <v>2026-09-04T07:13:08.637Z</v>
+        <v>2026-09-04T07:21:41.181Z</v>
       </c>
     </row>
     <row r="3">
@@ -639,10 +639,10 @@
         <v>Kích hoạt</v>
       </c>
       <c r="H3" t="str">
-        <v>$2b$10$gACgAHs317llVz7hBkSzueTGLnn6In3w1Fvzk0kANlfXI1qg4InL2</v>
+        <v>$2b$10$XSv.yrA1Pj8MUts1XMIYcuxvqv6rMCnq8C7kxgIp5j/tv1gZ4x4Fu</v>
       </c>
       <c r="I3" t="str">
-        <v>2026-09-04T07:13:08.637Z</v>
+        <v>2026-09-04T07:21:41.181Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>